<commit_message>
Normalize scenario workbooks: canonical headers, fix corruption + grammar + appliance names
- Rename all legacy headers to canonical snake_case (MANUAL_FOLLOWUP Part 1)
  across HVAC/Appliance/Shower/Test scenario + Appliance/Shower RAG files.
- Fix U+FFFD corruption (18 appliance master + 33 appliance RAG + 7 test cells):
  restore em-dash separators to match HVAC's legit em-dashes.
- Fix appliance question grammar: "It's just got home" -> "I've just got home".
- Canonicalize appliance values to {dishwasher,dryer,washing_machine}
  (washer->washing_machine, Dryer->dryer, Dishwasher->dishwasher) in master + RAG.
- Cell types unchanged (kept numeric per schema map; calculators coerce).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Scenario Files/ApplianceRAGScenarios.xlsx
+++ b/Scenario Files/ApplianceRAGScenarios.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>question</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>occupants</t>
+          <t>household_size</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>It's around 5 in the evening � when should I run the washing machine?</t>
+          <t>It's around 5 in the evening — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>It's around 5 in the evening � when should I run the washing machine?</t>
+          <t>It's around 5 in the evening — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>It's around 5 in the evening � when should I run the washing machine?</t>
+          <t>It's around 5 in the evening — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>It's just past 7 PM � when should I run the dryer?</t>
+          <t>It's just past 7 PM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>It's just past 7 PM � when should I run the dryer?</t>
+          <t>It's just past 7 PM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>It's just past 7 PM � when should I run the dryer?</t>
+          <t>It's just past 7 PM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>It's late � just past 10 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's late — just past 10 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>It's late � just past 10 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's late — just past 10 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>It's late � just past 10 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's late — just past 10 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>It's getting close to midnight � when should I run the washing machine?</t>
+          <t>It's getting close to midnight — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>It's getting close to midnight � when should I run the washing machine?</t>
+          <t>It's getting close to midnight — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>It's getting close to midnight � when should I run the washing machine?</t>
+          <t>It's getting close to midnight — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>It's just after 8 AM � when should I run the dishwasher?</t>
+          <t>It's just after 8 AM — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>It's just after 8 AM � when should I run the dishwasher?</t>
+          <t>It's just after 8 AM — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>It's just after 8 AM � when should I run the dishwasher?</t>
+          <t>It's just after 8 AM — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>It's nearly 11 at night � when should I run the washing machine?</t>
+          <t>It's nearly 11 at night — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>It's nearly 11 at night � when should I run the washing machine?</t>
+          <t>It's nearly 11 at night — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>It's nearly 11 at night � when should I run the washing machine?</t>
+          <t>It's nearly 11 at night — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>It's late afternoon, just past 3 � when should I run the dishwasher?</t>
+          <t>It's late afternoon, just past 3 — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -4738,7 +4738,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>It's late afternoon, just past 3 � when should I run the dishwasher?</t>
+          <t>It's late afternoon, just past 3 — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>It's late afternoon, just past 3 � when should I run the dishwasher?</t>
+          <t>It's late afternoon, just past 3 — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+          <t>It's around 2 in the afternoon — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+          <t>It's around 2 in the afternoon — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -6784,7 +6784,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+          <t>It's around 2 in the afternoon — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -6850,7 +6850,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
+          <t>I've just got home — it's around 6 PM — and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -6916,7 +6916,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
+          <t>I've just got home — it's around 6 PM — and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
+          <t>I've just got home — it's around 6 PM — and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -7061,7 +7061,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Dryer</t>
+          <t>dryer</t>
         </is>
       </c>
       <c r="F101" t="n">
@@ -7127,7 +7127,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Dryer</t>
+          <t>dryer</t>
         </is>
       </c>
       <c r="F102" t="n">
@@ -7193,7 +7193,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Dryer</t>
+          <t>dryer</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -7259,7 +7259,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Dishwasher</t>
+          <t>dishwasher</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -7325,7 +7325,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Dishwasher</t>
+          <t>dishwasher</t>
         </is>
       </c>
       <c r="F105" t="n">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Dishwasher</t>
+          <t>dishwasher</t>
         </is>
       </c>
       <c r="F106" t="n">

</xml_diff>

<commit_message>
Sync RAG scenario scores from regenerated ground truth
SyncRAGGroundTruth.py validation passed (descriptors match GT for every
(scenario_id, alternative) pair), then refreshed scores into the RAG corpus.
Partition unchanged: HVAC 35, Appliance 35, Shower 20 scenarios.
RAG files now carry canonical headers, fixed text, and current scores.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Scenario Files/ApplianceRAGScenarios.xlsx
+++ b/Scenario Files/ApplianceRAGScenarios.xlsx
@@ -530,8 +530,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>6</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -596,8 +598,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>6</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -662,8 +666,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>6</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -728,8 +734,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>8</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -794,8 +802,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>8</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -860,8 +870,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>8</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -926,8 +938,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>6</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -992,8 +1006,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>6</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1058,8 +1074,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>6</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1124,8 +1142,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>3</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1190,8 +1210,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>3</v>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1256,8 +1278,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>3</v>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1322,8 +1346,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>7</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1388,8 +1414,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>7</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1454,8 +1482,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>7</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1520,8 +1550,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>6</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1586,8 +1618,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>6</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1652,8 +1686,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>6</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1718,8 +1754,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>2</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1784,8 +1822,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>2</v>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1850,8 +1890,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>2</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1916,8 +1958,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>1</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1982,8 +2026,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>1</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2048,8 +2094,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>1</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2114,8 +2162,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>12</v>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2180,8 +2230,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>12</v>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -2246,8 +2298,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>12</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -2312,8 +2366,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>2</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -2378,8 +2434,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>2</v>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -2444,8 +2502,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>2</v>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -2510,8 +2570,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>6</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2576,8 +2638,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>6</v>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -2642,8 +2706,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F34" t="n">
-        <v>6</v>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -2708,8 +2774,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>5</v>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2774,8 +2842,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>5</v>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2840,8 +2910,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>5</v>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2906,8 +2978,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>7</v>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2972,8 +3046,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>7</v>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -3038,8 +3114,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F40" t="n">
-        <v>7</v>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -3104,8 +3182,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>5</v>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -3170,8 +3250,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F42" t="n">
-        <v>5</v>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -3236,8 +3318,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>5</v>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -3302,8 +3386,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F44" t="n">
-        <v>6</v>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -3368,8 +3454,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F45" t="n">
-        <v>6</v>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -3434,8 +3522,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F46" t="n">
-        <v>6</v>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -3500,8 +3590,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>6</v>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -3566,8 +3658,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F48" t="n">
-        <v>6</v>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -3632,8 +3726,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F49" t="n">
-        <v>6</v>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -3698,8 +3794,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F50" t="n">
-        <v>4</v>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -3764,8 +3862,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F51" t="n">
-        <v>4</v>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -3830,8 +3930,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F52" t="n">
-        <v>4</v>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -3896,8 +3998,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F53" t="n">
-        <v>1</v>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -3962,8 +4066,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F54" t="n">
-        <v>1</v>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -4028,8 +4134,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F55" t="n">
-        <v>1</v>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -4094,8 +4202,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F56" t="n">
-        <v>5</v>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -4160,8 +4270,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>5</v>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -4226,8 +4338,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F58" t="n">
-        <v>5</v>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -4292,8 +4406,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F59" t="n">
-        <v>6</v>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -4358,8 +4474,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F60" t="n">
-        <v>6</v>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -4424,8 +4542,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F61" t="n">
-        <v>6</v>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -4490,8 +4610,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F62" t="n">
-        <v>4</v>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -4556,8 +4678,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F63" t="n">
-        <v>4</v>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -4622,8 +4746,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F64" t="n">
-        <v>4</v>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -4688,8 +4814,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F65" t="n">
-        <v>6</v>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -4754,8 +4882,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F66" t="n">
-        <v>6</v>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -4820,8 +4950,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F67" t="n">
-        <v>6</v>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -4886,8 +5018,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F68" t="n">
-        <v>35</v>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -4952,8 +5086,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F69" t="n">
-        <v>35</v>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -5018,8 +5154,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F70" t="n">
-        <v>35</v>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -5084,8 +5222,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F71" t="n">
-        <v>38</v>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -5150,8 +5290,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F72" t="n">
-        <v>38</v>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -5216,8 +5358,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F73" t="n">
-        <v>38</v>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -5282,8 +5426,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F74" t="n">
-        <v>40</v>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -5348,8 +5494,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F75" t="n">
-        <v>40</v>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -5414,8 +5562,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F76" t="n">
-        <v>40</v>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -5480,8 +5630,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F77" t="n">
-        <v>7</v>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -5546,8 +5698,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F78" t="n">
-        <v>7</v>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -5612,8 +5766,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F79" t="n">
-        <v>7</v>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -5678,8 +5834,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F80" t="n">
-        <v>5</v>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -5744,8 +5902,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F81" t="n">
-        <v>5</v>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -5810,8 +5970,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F82" t="n">
-        <v>5</v>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -5876,8 +6038,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F83" t="n">
-        <v>9</v>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -5942,8 +6106,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F84" t="n">
-        <v>9</v>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -6008,8 +6174,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F85" t="n">
-        <v>9</v>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -6074,8 +6242,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F86" t="n">
-        <v>6</v>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -6140,8 +6310,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F87" t="n">
-        <v>6</v>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -6206,8 +6378,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F88" t="n">
-        <v>6</v>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -6272,8 +6446,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F89" t="n">
-        <v>8</v>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -6338,8 +6514,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F90" t="n">
-        <v>8</v>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -6404,8 +6582,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F91" t="n">
-        <v>8</v>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -6470,8 +6650,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F92" t="n">
-        <v>11</v>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -6536,8 +6718,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F93" t="n">
-        <v>11</v>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -6602,8 +6786,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F94" t="n">
-        <v>11</v>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -6668,8 +6854,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F95" t="n">
-        <v>7</v>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -6734,8 +6922,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F96" t="n">
-        <v>7</v>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -6800,8 +6990,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F97" t="n">
-        <v>7</v>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -6866,8 +7058,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F98" t="n">
-        <v>10</v>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -6932,8 +7126,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F99" t="n">
-        <v>10</v>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -6998,8 +7194,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F100" t="n">
-        <v>10</v>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -7064,8 +7262,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F101" t="n">
-        <v>9</v>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -7130,8 +7330,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F102" t="n">
-        <v>9</v>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -7196,8 +7398,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F103" t="n">
-        <v>9</v>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -7262,8 +7466,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F104" t="n">
-        <v>6</v>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -7328,8 +7534,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F105" t="n">
-        <v>6</v>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -7394,8 +7602,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F106" t="n">
-        <v>6</v>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
updated keys, ran qwen and deepseek to test reasoning fixces. also converted the RAG to 0-1 range.
</commit_message>
<xml_diff>
--- a/Scenario Files/ApplianceRAGScenarios.xlsx
+++ b/Scenario Files/ApplianceRAGScenarios.xlsx
@@ -552,19 +552,19 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>6.56</v>
+        <v>0.66</v>
       </c>
       <c r="L2" t="n">
-        <v>2.17</v>
+        <v>0.22</v>
       </c>
       <c r="M2" t="n">
-        <v>9.460000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="N2" t="n">
-        <v>9.15</v>
+        <v>0.91</v>
       </c>
       <c r="O2" t="n">
-        <v>5.992000000000001</v>
+        <v>0.6015</v>
       </c>
       <c r="P2" t="n">
         <v>1</v>
@@ -620,19 +620,19 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>6.56</v>
+        <v>0.66</v>
       </c>
       <c r="L3" t="n">
-        <v>2.17</v>
+        <v>0.22</v>
       </c>
       <c r="M3" t="n">
-        <v>8.9</v>
+        <v>0.89</v>
       </c>
       <c r="N3" t="n">
-        <v>8.23</v>
+        <v>0.82</v>
       </c>
       <c r="O3" t="n">
-        <v>5.742</v>
+        <v>0.5760000000000001</v>
       </c>
       <c r="P3" t="n">
         <v>2</v>
@@ -688,19 +688,19 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2.8</v>
+        <v>0.28</v>
       </c>
       <c r="L4" t="n">
-        <v>2.17</v>
+        <v>0.22</v>
       </c>
       <c r="M4" t="n">
-        <v>6.74</v>
+        <v>0.67</v>
       </c>
       <c r="N4" t="n">
-        <v>5.4</v>
+        <v>0.54</v>
       </c>
       <c r="O4" t="n">
-        <v>3.7575</v>
+        <v>0.3760000000000001</v>
       </c>
       <c r="P4" t="n">
         <v>3</v>
@@ -756,19 +756,19 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>5.61</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>5.183</v>
+        <v>0.518</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
@@ -824,19 +824,19 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>5.61</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>7.81</v>
+        <v>0.78</v>
       </c>
       <c r="N6" t="n">
-        <v>6.66</v>
+        <v>0.67</v>
       </c>
       <c r="O6" t="n">
-        <v>4.244</v>
+        <v>0.4245000000000001</v>
       </c>
       <c r="P6" t="n">
         <v>2</v>
@@ -892,19 +892,19 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>0.91</v>
+        <v>0.09</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>5.92</v>
+        <v>0.59</v>
       </c>
       <c r="N7" t="n">
-        <v>4.31</v>
+        <v>0.43</v>
       </c>
       <c r="O7" t="n">
-        <v>2.1035</v>
+        <v>0.2095</v>
       </c>
       <c r="P7" t="n">
         <v>3</v>
@@ -960,19 +960,19 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>9.77</v>
+        <v>0.98</v>
       </c>
       <c r="M8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O8" t="n">
-        <v>9.919499999999999</v>
+        <v>0.993</v>
       </c>
       <c r="P8" t="n">
         <v>1</v>
@@ -1028,19 +1028,19 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>9.550000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="L9" t="n">
-        <v>9.77</v>
+        <v>0.98</v>
       </c>
       <c r="M9" t="n">
-        <v>6.92</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="N9" t="n">
-        <v>5.61</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="O9" t="n">
-        <v>8.51</v>
+        <v>0.8499999999999999</v>
       </c>
       <c r="P9" t="n">
         <v>2</v>
@@ -1096,19 +1096,19 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>9.84</v>
+        <v>0.98</v>
       </c>
       <c r="M10" t="n">
-        <v>3.83</v>
+        <v>0.38</v>
       </c>
       <c r="N10" t="n">
-        <v>1.51</v>
+        <v>0.15</v>
       </c>
       <c r="O10" t="n">
-        <v>7.4365</v>
+        <v>0.7415</v>
       </c>
       <c r="P10" t="n">
         <v>3</v>
@@ -1164,19 +1164,19 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>9.140000000000001</v>
+        <v>0.91</v>
       </c>
       <c r="L11" t="n">
-        <v>7.45</v>
+        <v>0.74</v>
       </c>
       <c r="M11" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N11" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O11" t="n">
-        <v>8.849499999999999</v>
+        <v>0.882</v>
       </c>
       <c r="P11" t="n">
         <v>1</v>
@@ -1232,19 +1232,19 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>5.23</v>
+        <v>0.52</v>
       </c>
       <c r="L12" t="n">
-        <v>7.45</v>
+        <v>0.74</v>
       </c>
       <c r="M12" t="n">
-        <v>7.83</v>
+        <v>0.78</v>
       </c>
       <c r="N12" t="n">
-        <v>6.69</v>
+        <v>0.67</v>
       </c>
       <c r="O12" t="n">
-        <v>6.746</v>
+        <v>0.6715000000000001</v>
       </c>
       <c r="P12" t="n">
         <v>3</v>
@@ -1300,19 +1300,19 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>9.140000000000001</v>
+        <v>0.91</v>
       </c>
       <c r="L13" t="n">
-        <v>7.45</v>
+        <v>0.74</v>
       </c>
       <c r="M13" t="n">
-        <v>6.29</v>
+        <v>0.63</v>
       </c>
       <c r="N13" t="n">
-        <v>4.78</v>
+        <v>0.48</v>
       </c>
       <c r="O13" t="n">
-        <v>7.3245</v>
+        <v>0.73</v>
       </c>
       <c r="P13" t="n">
         <v>2</v>
@@ -1368,19 +1368,19 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>9.91</v>
+        <v>0.99</v>
       </c>
       <c r="L14" t="n">
-        <v>9.460000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="M14" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N14" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>9.783999999999999</v>
+        <v>0.9794999999999999</v>
       </c>
       <c r="P14" t="n">
         <v>1</v>
@@ -1436,19 +1436,19 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>9.91</v>
+        <v>0.99</v>
       </c>
       <c r="L15" t="n">
-        <v>9.460000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="M15" t="n">
-        <v>4.71</v>
+        <v>0.47</v>
       </c>
       <c r="N15" t="n">
-        <v>2.95</v>
+        <v>0.3</v>
       </c>
       <c r="O15" t="n">
-        <v>7.6685</v>
+        <v>0.7685</v>
       </c>
       <c r="P15" t="n">
         <v>2</v>
@@ -1504,19 +1504,19 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>9.91</v>
+        <v>0.99</v>
       </c>
       <c r="L16" t="n">
-        <v>9.550000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="M16" t="n">
-        <v>2.86</v>
+        <v>0.29</v>
       </c>
       <c r="N16" t="n">
-        <v>1.51</v>
+        <v>0.15</v>
       </c>
       <c r="O16" t="n">
-        <v>7.114</v>
+        <v>0.71</v>
       </c>
       <c r="P16" t="n">
         <v>3</v>
@@ -1572,19 +1572,19 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>4.74</v>
+        <v>0.47</v>
       </c>
       <c r="L17" t="n">
-        <v>2.17</v>
+        <v>0.22</v>
       </c>
       <c r="M17" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N17" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O17" t="n">
-        <v>5.6815</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="P17" t="n">
         <v>1</v>
@@ -1640,19 +1640,19 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>4.74</v>
+        <v>0.47</v>
       </c>
       <c r="L18" t="n">
-        <v>2.17</v>
+        <v>0.22</v>
       </c>
       <c r="M18" t="n">
-        <v>7.29</v>
+        <v>0.73</v>
       </c>
       <c r="N18" t="n">
-        <v>6.04</v>
+        <v>0.6</v>
       </c>
       <c r="O18" t="n">
-        <v>4.5455</v>
+        <v>0.454</v>
       </c>
       <c r="P18" t="n">
         <v>2</v>
@@ -1708,19 +1708,19 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>4.74</v>
+        <v>0.47</v>
       </c>
       <c r="L19" t="n">
-        <v>2.71</v>
+        <v>0.27</v>
       </c>
       <c r="M19" t="n">
-        <v>2.35</v>
+        <v>0.23</v>
       </c>
       <c r="N19" t="n">
-        <v>2.13</v>
+        <v>0.21</v>
       </c>
       <c r="O19" t="n">
-        <v>3.16</v>
+        <v>0.3129999999999999</v>
       </c>
       <c r="P19" t="n">
         <v>3</v>
@@ -1776,19 +1776,19 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>9.9</v>
+        <v>0.99</v>
       </c>
       <c r="L20" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N20" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O20" t="n">
-        <v>9.970000000000001</v>
+        <v>0.997</v>
       </c>
       <c r="P20" t="n">
         <v>1</v>
@@ -1844,19 +1844,19 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>7</v>
+        <v>0.7</v>
       </c>
       <c r="N21" t="n">
-        <v>5.71</v>
+        <v>0.57</v>
       </c>
       <c r="O21" t="n">
-        <v>8.756500000000001</v>
+        <v>0.8754999999999999</v>
       </c>
       <c r="P21" t="n">
         <v>2</v>
@@ -1912,19 +1912,19 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L22" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>3.59</v>
+        <v>0.36</v>
       </c>
       <c r="N22" t="n">
-        <v>2.86</v>
+        <v>0.29</v>
       </c>
       <c r="O22" t="n">
-        <v>7.647</v>
+        <v>0.7654999999999998</v>
       </c>
       <c r="P22" t="n">
         <v>3</v>
@@ -1980,19 +1980,19 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>9.83</v>
+        <v>0.98</v>
       </c>
       <c r="L23" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N23" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O23" t="n">
-        <v>9.949</v>
+        <v>0.9939999999999999</v>
       </c>
       <c r="P23" t="n">
         <v>1</v>
@@ -2048,19 +2048,19 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>5.92</v>
+        <v>0.59</v>
       </c>
       <c r="N24" t="n">
-        <v>4.64</v>
+        <v>0.43</v>
       </c>
       <c r="O24" t="n">
-        <v>8.380000000000001</v>
+        <v>0.8324999999999999</v>
       </c>
       <c r="P24" t="n">
         <v>3</v>
@@ -2116,19 +2116,19 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>6.01</v>
+        <v>0.6</v>
       </c>
       <c r="N25" t="n">
-        <v>5.19</v>
+        <v>0.52</v>
       </c>
       <c r="O25" t="n">
-        <v>8.480499999999999</v>
+        <v>0.8479999999999999</v>
       </c>
       <c r="P25" t="n">
         <v>2</v>
@@ -2184,19 +2184,19 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>6.79</v>
+        <v>0.68</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N26" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O26" t="n">
-        <v>5.537</v>
+        <v>0.554</v>
       </c>
       <c r="P26" t="n">
         <v>1</v>
@@ -2252,19 +2252,19 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>6.79</v>
+        <v>0.68</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>5.13</v>
+        <v>0.51</v>
       </c>
       <c r="N27" t="n">
-        <v>3.42</v>
+        <v>0.34</v>
       </c>
       <c r="O27" t="n">
-        <v>3.576</v>
+        <v>0.357</v>
       </c>
       <c r="P27" t="n">
         <v>3</v>
@@ -2320,19 +2320,19 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>6.79</v>
+        <v>0.68</v>
       </c>
       <c r="L28" t="n">
-        <v>0.68</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="M28" t="n">
-        <v>5.06</v>
+        <v>0.51</v>
       </c>
       <c r="N28" t="n">
-        <v>3.88</v>
+        <v>0.39</v>
       </c>
       <c r="O28" t="n">
-        <v>3.869</v>
+        <v>0.389</v>
       </c>
       <c r="P28" t="n">
         <v>2</v>
@@ -2388,19 +2388,19 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>7</v>
+        <v>0.7</v>
       </c>
       <c r="L29" t="n">
-        <v>8.619999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="M29" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O29" t="n">
-        <v>8.616999999999999</v>
+        <v>0.8610000000000001</v>
       </c>
       <c r="P29" t="n">
         <v>1</v>
@@ -2456,19 +2456,19 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>9.57</v>
+        <v>0.96</v>
       </c>
       <c r="L30" t="n">
-        <v>8.619999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="M30" t="n">
-        <v>7.43</v>
+        <v>0.74</v>
       </c>
       <c r="N30" t="n">
-        <v>6.21</v>
+        <v>0.62</v>
       </c>
       <c r="O30" t="n">
-        <v>8.3055</v>
+        <v>0.83</v>
       </c>
       <c r="P30" t="n">
         <v>2</v>
@@ -2524,19 +2524,19 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>9.57</v>
+        <v>0.96</v>
       </c>
       <c r="L31" t="n">
-        <v>8.619999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="M31" t="n">
-        <v>7</v>
+        <v>0.7</v>
       </c>
       <c r="N31" t="n">
-        <v>4.64</v>
+        <v>0.46</v>
       </c>
       <c r="O31" t="n">
-        <v>7.984</v>
+        <v>0.798</v>
       </c>
       <c r="P31" t="n">
         <v>3</v>
@@ -2592,19 +2592,19 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>7.59</v>
+        <v>0.76</v>
       </c>
       <c r="L32" t="n">
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M32" t="n">
-        <v>7.83</v>
+        <v>0.78</v>
       </c>
       <c r="N32" t="n">
-        <v>9.25</v>
+        <v>0.93</v>
       </c>
       <c r="O32" t="n">
-        <v>6.3155</v>
+        <v>0.632</v>
       </c>
       <c r="P32" t="n">
         <v>1</v>
@@ -2660,19 +2660,19 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>7.59</v>
+        <v>0.76</v>
       </c>
       <c r="L33" t="n">
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M33" t="n">
-        <v>4.71</v>
+        <v>0.47</v>
       </c>
       <c r="N33" t="n">
-        <v>2.95</v>
+        <v>0.3</v>
       </c>
       <c r="O33" t="n">
-        <v>4.746499999999999</v>
+        <v>0.4755</v>
       </c>
       <c r="P33" t="n">
         <v>2</v>
@@ -2731,16 +2731,16 @@
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M34" t="n">
-        <v>5.92</v>
+        <v>0.59</v>
       </c>
       <c r="N34" t="n">
-        <v>4.31</v>
+        <v>0.43</v>
       </c>
       <c r="O34" t="n">
-        <v>2.9155</v>
+        <v>0.291</v>
       </c>
       <c r="P34" t="n">
         <v>3</v>
@@ -2796,19 +2796,19 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>9.789999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="L35" t="n">
-        <v>9.550000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="M35" t="n">
-        <v>8.300000000000001</v>
+        <v>0.83</v>
       </c>
       <c r="N35" t="n">
-        <v>9.25</v>
+        <v>0.93</v>
       </c>
       <c r="O35" t="n">
-        <v>9.327</v>
+        <v>0.9319999999999999</v>
       </c>
       <c r="P35" t="n">
         <v>1</v>
@@ -2864,22 +2864,22 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>9.789999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="L36" t="n">
-        <v>9.460000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="M36" t="n">
-        <v>5.53</v>
+        <v>0.55</v>
       </c>
       <c r="N36" t="n">
-        <v>3.87</v>
+        <v>0.39</v>
       </c>
       <c r="O36" t="n">
-        <v>7.934499999999999</v>
+        <v>0.7949999999999999</v>
       </c>
       <c r="P36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q36" t="n">
         <v>0.0396</v>
@@ -2932,22 +2932,22 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>9.24</v>
+        <v>0.92</v>
       </c>
       <c r="L37" t="n">
-        <v>9.460000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="M37" t="n">
-        <v>5.92</v>
+        <v>0.59</v>
       </c>
       <c r="N37" t="n">
-        <v>4.64</v>
+        <v>0.43</v>
       </c>
       <c r="O37" t="n">
-        <v>7.963</v>
+        <v>0.791</v>
       </c>
       <c r="P37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q37" t="n">
         <v>0.0774</v>
@@ -3000,19 +3000,19 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>4.53</v>
+        <v>0.45</v>
       </c>
       <c r="L38" t="n">
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M38" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N38" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O38" t="n">
-        <v>5.944</v>
+        <v>0.5935</v>
       </c>
       <c r="P38" t="n">
         <v>1</v>
@@ -3068,19 +3068,19 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>4.53</v>
+        <v>0.45</v>
       </c>
       <c r="L39" t="n">
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M39" t="n">
-        <v>8.73</v>
+        <v>0.87</v>
       </c>
       <c r="N39" t="n">
-        <v>8.029999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="O39" t="n">
-        <v>5.394500000000001</v>
+        <v>0.5375</v>
       </c>
       <c r="P39" t="n">
         <v>2</v>
@@ -3136,19 +3136,19 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>7.81</v>
+        <v>0.78</v>
       </c>
       <c r="L40" t="n">
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M40" t="n">
-        <v>6.11</v>
+        <v>0.61</v>
       </c>
       <c r="N40" t="n">
-        <v>4.64</v>
+        <v>0.46</v>
       </c>
       <c r="O40" t="n">
-        <v>5.346</v>
+        <v>0.5335</v>
       </c>
       <c r="P40" t="n">
         <v>3</v>
@@ -3204,19 +3204,19 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>9.24</v>
+        <v>0.92</v>
       </c>
       <c r="L41" t="n">
-        <v>7.45</v>
+        <v>0.74</v>
       </c>
       <c r="M41" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N41" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O41" t="n">
-        <v>8.8795</v>
+        <v>0.8850000000000001</v>
       </c>
       <c r="P41" t="n">
         <v>1</v>
@@ -3272,19 +3272,19 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>7.8</v>
+        <v>0.78</v>
       </c>
       <c r="L42" t="n">
-        <v>7.45</v>
+        <v>0.74</v>
       </c>
       <c r="M42" t="n">
-        <v>7.09</v>
+        <v>0.71</v>
       </c>
       <c r="N42" t="n">
-        <v>5.81</v>
+        <v>0.58</v>
       </c>
       <c r="O42" t="n">
-        <v>7.237</v>
+        <v>0.722</v>
       </c>
       <c r="P42" t="n">
         <v>2</v>
@@ -3340,19 +3340,19 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>9.24</v>
+        <v>0.92</v>
       </c>
       <c r="L43" t="n">
-        <v>7.45</v>
+        <v>0.74</v>
       </c>
       <c r="M43" t="n">
-        <v>4.78</v>
+        <v>0.48</v>
       </c>
       <c r="N43" t="n">
-        <v>4.64</v>
+        <v>0.3</v>
       </c>
       <c r="O43" t="n">
-        <v>7.0315</v>
+        <v>0.676</v>
       </c>
       <c r="P43" t="n">
         <v>3</v>
@@ -3408,19 +3408,19 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>9.98</v>
+        <v>1</v>
       </c>
       <c r="L44" t="n">
-        <v>9.75</v>
+        <v>0.98</v>
       </c>
       <c r="M44" t="n">
-        <v>7.83</v>
+        <v>0.78</v>
       </c>
       <c r="N44" t="n">
-        <v>8.449999999999999</v>
+        <v>0.85</v>
       </c>
       <c r="O44" t="n">
-        <v>9.239999999999998</v>
+        <v>0.9265000000000001</v>
       </c>
       <c r="P44" t="n">
         <v>1</v>
@@ -3476,19 +3476,19 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>9.98</v>
+        <v>1</v>
       </c>
       <c r="L45" t="n">
-        <v>9.68</v>
+        <v>0.97</v>
       </c>
       <c r="M45" t="n">
-        <v>5.23</v>
+        <v>0.52</v>
       </c>
       <c r="N45" t="n">
-        <v>4.64</v>
+        <v>0.35</v>
       </c>
       <c r="O45" t="n">
-        <v>8.124000000000001</v>
+        <v>0.7959999999999999</v>
       </c>
       <c r="P45" t="n">
         <v>2</v>
@@ -3544,19 +3544,19 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>9.48</v>
+        <v>0.95</v>
       </c>
       <c r="L46" t="n">
-        <v>9.68</v>
+        <v>0.97</v>
       </c>
       <c r="M46" t="n">
-        <v>3.94</v>
+        <v>0.39</v>
       </c>
       <c r="N46" t="n">
-        <v>2.03</v>
+        <v>0.2</v>
       </c>
       <c r="O46" t="n">
-        <v>7.3245</v>
+        <v>0.7324999999999999</v>
       </c>
       <c r="P46" t="n">
         <v>3</v>
@@ -3612,19 +3612,19 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>6.72</v>
+        <v>0.67</v>
       </c>
       <c r="L47" t="n">
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M47" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N47" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O47" t="n">
-        <v>6.601</v>
+        <v>0.6595000000000001</v>
       </c>
       <c r="P47" t="n">
         <v>1</v>
@@ -3680,19 +3680,19 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>2.96</v>
+        <v>0.3</v>
       </c>
       <c r="L48" t="n">
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M48" t="n">
-        <v>7.81</v>
+        <v>0.78</v>
       </c>
       <c r="N48" t="n">
-        <v>6.66</v>
+        <v>0.67</v>
       </c>
       <c r="O48" t="n">
-        <v>4.534</v>
+        <v>0.4550000000000001</v>
       </c>
       <c r="P48" t="n">
         <v>2</v>
@@ -3748,19 +3748,19 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>6.72</v>
+        <v>0.67</v>
       </c>
       <c r="L49" t="n">
-        <v>3.59</v>
+        <v>0.36</v>
       </c>
       <c r="M49" t="n">
-        <v>2.86</v>
+        <v>0.29</v>
       </c>
       <c r="N49" t="n">
-        <v>1.51</v>
+        <v>0.15</v>
       </c>
       <c r="O49" t="n">
-        <v>4.071</v>
+        <v>0.4075</v>
       </c>
       <c r="P49" t="n">
         <v>3</v>
@@ -3816,19 +3816,19 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>9.9</v>
+        <v>0.99</v>
       </c>
       <c r="L50" t="n">
-        <v>9.869999999999999</v>
+        <v>0.99</v>
       </c>
       <c r="M50" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N50" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O50" t="n">
-        <v>9.9245</v>
+        <v>0.9934999999999999</v>
       </c>
       <c r="P50" t="n">
         <v>1</v>
@@ -3884,19 +3884,19 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>9.42</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L51" t="n">
-        <v>9.869999999999999</v>
+        <v>0.99</v>
       </c>
       <c r="M51" t="n">
-        <v>7.43</v>
+        <v>0.74</v>
       </c>
       <c r="N51" t="n">
-        <v>6.21</v>
+        <v>0.62</v>
       </c>
       <c r="O51" t="n">
-        <v>8.698</v>
+        <v>0.8694999999999999</v>
       </c>
       <c r="P51" t="n">
         <v>2</v>
@@ -3952,19 +3952,19 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>9.9</v>
+        <v>0.99</v>
       </c>
       <c r="L52" t="n">
-        <v>9.869999999999999</v>
+        <v>0.99</v>
       </c>
       <c r="M52" t="n">
-        <v>1.53</v>
+        <v>0.15</v>
       </c>
       <c r="N52" t="n">
-        <v>2.2</v>
+        <v>0.22</v>
       </c>
       <c r="O52" t="n">
-        <v>7.0605</v>
+        <v>0.7065</v>
       </c>
       <c r="P52" t="n">
         <v>3</v>
@@ -4020,19 +4020,19 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>9.66</v>
+        <v>0.97</v>
       </c>
       <c r="L53" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M53" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N53" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O53" t="n">
-        <v>9.898</v>
+        <v>0.991</v>
       </c>
       <c r="P53" t="n">
         <v>1</v>
@@ -4088,19 +4088,19 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L54" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M54" t="n">
-        <v>7.43</v>
+        <v>0.74</v>
       </c>
       <c r="N54" t="n">
-        <v>6.21</v>
+        <v>0.62</v>
       </c>
       <c r="O54" t="n">
-        <v>8.9175</v>
+        <v>0.8909999999999999</v>
       </c>
       <c r="P54" t="n">
         <v>2</v>
@@ -4156,19 +4156,19 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L55" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M55" t="n">
-        <v>3.59</v>
+        <v>0.36</v>
       </c>
       <c r="N55" t="n">
-        <v>4.08</v>
+        <v>0.41</v>
       </c>
       <c r="O55" t="n">
-        <v>7.83</v>
+        <v>0.7834999999999999</v>
       </c>
       <c r="P55" t="n">
         <v>3</v>
@@ -4224,19 +4224,19 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>5.35</v>
+        <v>0.53</v>
       </c>
       <c r="L56" t="n">
-        <v>3.59</v>
+        <v>0.36</v>
       </c>
       <c r="M56" t="n">
-        <v>7.83</v>
+        <v>0.78</v>
       </c>
       <c r="N56" t="n">
-        <v>8.449999999999999</v>
+        <v>0.85</v>
       </c>
       <c r="O56" t="n">
-        <v>5.694999999999999</v>
+        <v>0.5685</v>
       </c>
       <c r="P56" t="n">
         <v>1</v>
@@ -4292,19 +4292,19 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>5.35</v>
+        <v>0.53</v>
       </c>
       <c r="L57" t="n">
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M57" t="n">
-        <v>5.53</v>
+        <v>0.55</v>
       </c>
       <c r="N57" t="n">
-        <v>3.87</v>
+        <v>0.39</v>
       </c>
       <c r="O57" t="n">
-        <v>4.376499999999999</v>
+        <v>0.4360000000000001</v>
       </c>
       <c r="P57" t="n">
         <v>2</v>
@@ -4360,19 +4360,19 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>5.35</v>
+        <v>0.53</v>
       </c>
       <c r="L58" t="n">
-        <v>3.1</v>
+        <v>0.31</v>
       </c>
       <c r="M58" t="n">
-        <v>5.13</v>
+        <v>0.51</v>
       </c>
       <c r="N58" t="n">
-        <v>3.42</v>
+        <v>0.34</v>
       </c>
       <c r="O58" t="n">
-        <v>4.228999999999999</v>
+        <v>0.4205</v>
       </c>
       <c r="P58" t="n">
         <v>3</v>
@@ -4428,19 +4428,19 @@
         </is>
       </c>
       <c r="K59" t="n">
-        <v>9.789999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="L59" t="n">
-        <v>9.640000000000001</v>
+        <v>0.96</v>
       </c>
       <c r="M59" t="n">
-        <v>7.83</v>
+        <v>0.78</v>
       </c>
       <c r="N59" t="n">
-        <v>9.25</v>
+        <v>0.93</v>
       </c>
       <c r="O59" t="n">
-        <v>9.2645</v>
+        <v>0.9255</v>
       </c>
       <c r="P59" t="n">
         <v>1</v>
@@ -4496,19 +4496,19 @@
         </is>
       </c>
       <c r="K60" t="n">
-        <v>9.789999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="L60" t="n">
-        <v>9.56</v>
+        <v>0.96</v>
       </c>
       <c r="M60" t="n">
-        <v>4.71</v>
+        <v>0.47</v>
       </c>
       <c r="N60" t="n">
-        <v>2.95</v>
+        <v>0.3</v>
       </c>
       <c r="O60" t="n">
-        <v>7.6675</v>
+        <v>0.7689999999999999</v>
       </c>
       <c r="P60" t="n">
         <v>3</v>
@@ -4564,19 +4564,19 @@
         </is>
       </c>
       <c r="K61" t="n">
-        <v>9.23</v>
+        <v>0.92</v>
       </c>
       <c r="L61" t="n">
-        <v>9.56</v>
+        <v>0.96</v>
       </c>
       <c r="M61" t="n">
-        <v>5.92</v>
+        <v>0.59</v>
       </c>
       <c r="N61" t="n">
-        <v>4.64</v>
+        <v>0.43</v>
       </c>
       <c r="O61" t="n">
-        <v>7.995</v>
+        <v>0.7945</v>
       </c>
       <c r="P61" t="n">
         <v>2</v>
@@ -4632,19 +4632,19 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>9.029999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="L62" t="n">
-        <v>7.37</v>
+        <v>0.74</v>
       </c>
       <c r="M62" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N62" t="n">
-        <v>8.449999999999999</v>
+        <v>0.85</v>
       </c>
       <c r="O62" t="n">
-        <v>8.555999999999999</v>
+        <v>0.8565</v>
       </c>
       <c r="P62" t="n">
         <v>1</v>
@@ -4700,19 +4700,19 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>9.029999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="L63" t="n">
-        <v>7.14</v>
+        <v>0.71</v>
       </c>
       <c r="M63" t="n">
-        <v>8.02</v>
+        <v>0.8</v>
       </c>
       <c r="N63" t="n">
-        <v>6.91</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="O63" t="n">
-        <v>7.8485</v>
+        <v>0.782</v>
       </c>
       <c r="P63" t="n">
         <v>2</v>
@@ -4768,19 +4768,19 @@
         </is>
       </c>
       <c r="K64" t="n">
-        <v>9.029999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="L64" t="n">
-        <v>7.14</v>
+        <v>0.71</v>
       </c>
       <c r="M64" t="n">
-        <v>5.26</v>
+        <v>0.53</v>
       </c>
       <c r="N64" t="n">
-        <v>4.64</v>
+        <v>0.36</v>
       </c>
       <c r="O64" t="n">
-        <v>6.956</v>
+        <v>0.6785</v>
       </c>
       <c r="P64" t="n">
         <v>3</v>
@@ -4836,19 +4836,19 @@
         </is>
       </c>
       <c r="K65" t="n">
-        <v>7.73</v>
+        <v>0.77</v>
       </c>
       <c r="L65" t="n">
-        <v>7.6</v>
+        <v>0.76</v>
       </c>
       <c r="M65" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N65" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O65" t="n">
-        <v>8.478999999999999</v>
+        <v>0.847</v>
       </c>
       <c r="P65" t="n">
         <v>1</v>
@@ -4904,19 +4904,19 @@
         </is>
       </c>
       <c r="K66" t="n">
-        <v>9.02</v>
+        <v>0.9</v>
       </c>
       <c r="L66" t="n">
-        <v>7.6</v>
+        <v>0.76</v>
       </c>
       <c r="M66" t="n">
-        <v>7.09</v>
+        <v>0.71</v>
       </c>
       <c r="N66" t="n">
-        <v>5.81</v>
+        <v>0.58</v>
       </c>
       <c r="O66" t="n">
-        <v>7.6555</v>
+        <v>0.765</v>
       </c>
       <c r="P66" t="n">
         <v>2</v>
@@ -4972,19 +4972,19 @@
         </is>
       </c>
       <c r="K67" t="n">
-        <v>9.02</v>
+        <v>0.9</v>
       </c>
       <c r="L67" t="n">
-        <v>7.8</v>
+        <v>0.78</v>
       </c>
       <c r="M67" t="n">
-        <v>6.17</v>
+        <v>0.62</v>
       </c>
       <c r="N67" t="n">
-        <v>3.44</v>
+        <v>0.34</v>
       </c>
       <c r="O67" t="n">
-        <v>7.186</v>
+        <v>0.718</v>
       </c>
       <c r="P67" t="n">
         <v>3</v>
@@ -5040,19 +5040,19 @@
         </is>
       </c>
       <c r="K68" t="n">
-        <v>6.65</v>
+        <v>0.67</v>
       </c>
       <c r="L68" t="n">
-        <v>5.12</v>
+        <v>0.51</v>
       </c>
       <c r="M68" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N68" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O68" t="n">
-        <v>7.287</v>
+        <v>0.7295</v>
       </c>
       <c r="P68" t="n">
         <v>1</v>
@@ -5108,19 +5108,19 @@
         </is>
       </c>
       <c r="K69" t="n">
-        <v>6.65</v>
+        <v>0.67</v>
       </c>
       <c r="L69" t="n">
-        <v>5.12</v>
+        <v>0.51</v>
       </c>
       <c r="M69" t="n">
-        <v>7.09</v>
+        <v>0.71</v>
       </c>
       <c r="N69" t="n">
-        <v>5.81</v>
+        <v>0.58</v>
       </c>
       <c r="O69" t="n">
-        <v>6.0765</v>
+        <v>0.6084999999999999</v>
       </c>
       <c r="P69" t="n">
         <v>2</v>
@@ -5176,19 +5176,19 @@
         </is>
       </c>
       <c r="K70" t="n">
-        <v>6.65</v>
+        <v>0.67</v>
       </c>
       <c r="L70" t="n">
-        <v>5.48</v>
+        <v>0.55</v>
       </c>
       <c r="M70" t="n">
-        <v>5.73</v>
+        <v>0.57</v>
       </c>
       <c r="N70" t="n">
-        <v>2.89</v>
+        <v>0.29</v>
       </c>
       <c r="O70" t="n">
-        <v>5.4925</v>
+        <v>0.551</v>
       </c>
       <c r="P70" t="n">
         <v>3</v>
@@ -5250,13 +5250,13 @@
         <v>0</v>
       </c>
       <c r="M71" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N71" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O71" t="n">
-        <v>3.5</v>
+        <v>0.35</v>
       </c>
       <c r="P71" t="n">
         <v>1</v>
@@ -5312,19 +5312,19 @@
         </is>
       </c>
       <c r="K72" t="n">
-        <v>4.8</v>
+        <v>0.48</v>
       </c>
       <c r="L72" t="n">
         <v>0</v>
       </c>
       <c r="M72" t="n">
-        <v>6.29</v>
+        <v>0.63</v>
       </c>
       <c r="N72" t="n">
-        <v>4.86</v>
+        <v>0.49</v>
       </c>
       <c r="O72" t="n">
-        <v>3.427</v>
+        <v>0.3435</v>
       </c>
       <c r="P72" t="n">
         <v>2</v>
@@ -5380,19 +5380,19 @@
         </is>
       </c>
       <c r="K73" t="n">
-        <v>4.8</v>
+        <v>0.48</v>
       </c>
       <c r="L73" t="n">
         <v>0</v>
       </c>
       <c r="M73" t="n">
-        <v>1.24</v>
+        <v>0.12</v>
       </c>
       <c r="N73" t="n">
-        <v>1.51</v>
+        <v>0.15</v>
       </c>
       <c r="O73" t="n">
-        <v>1.9145</v>
+        <v>0.1905</v>
       </c>
       <c r="P73" t="n">
         <v>3</v>
@@ -5448,19 +5448,19 @@
         </is>
       </c>
       <c r="K74" t="n">
-        <v>8.220000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="L74" t="n">
-        <v>4.34</v>
+        <v>0.43</v>
       </c>
       <c r="M74" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N74" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O74" t="n">
-        <v>7.485</v>
+        <v>0.7465000000000001</v>
       </c>
       <c r="P74" t="n">
         <v>1</v>
@@ -5516,19 +5516,19 @@
         </is>
       </c>
       <c r="K75" t="n">
-        <v>5.46</v>
+        <v>0.55</v>
       </c>
       <c r="L75" t="n">
-        <v>4.34</v>
+        <v>0.43</v>
       </c>
       <c r="M75" t="n">
-        <v>8.02</v>
+        <v>0.8</v>
       </c>
       <c r="N75" t="n">
-        <v>6.91</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="O75" t="n">
-        <v>5.7975</v>
+        <v>0.5790000000000001</v>
       </c>
       <c r="P75" t="n">
         <v>2</v>
@@ -5584,19 +5584,19 @@
         </is>
       </c>
       <c r="K76" t="n">
-        <v>8.220000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="L76" t="n">
-        <v>4.75</v>
+        <v>0.47</v>
       </c>
       <c r="M76" t="n">
-        <v>4.78</v>
+        <v>0.48</v>
       </c>
       <c r="N76" t="n">
-        <v>1.71</v>
+        <v>0.17</v>
       </c>
       <c r="O76" t="n">
-        <v>5.341</v>
+        <v>0.5319999999999999</v>
       </c>
       <c r="P76" t="n">
         <v>3</v>
@@ -5652,19 +5652,19 @@
         </is>
       </c>
       <c r="K77" t="n">
-        <v>4.99</v>
+        <v>0.5</v>
       </c>
       <c r="L77" t="n">
-        <v>7.29</v>
+        <v>0.73</v>
       </c>
       <c r="M77" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N77" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O77" t="n">
-        <v>7.5485</v>
+        <v>0.7554999999999999</v>
       </c>
       <c r="P77" t="n">
         <v>2</v>
@@ -5720,19 +5720,19 @@
         </is>
       </c>
       <c r="K78" t="n">
-        <v>9.09</v>
+        <v>0.91</v>
       </c>
       <c r="L78" t="n">
-        <v>7.51</v>
+        <v>0.75</v>
       </c>
       <c r="M78" t="n">
-        <v>7.43</v>
+        <v>0.74</v>
       </c>
       <c r="N78" t="n">
-        <v>5.19</v>
+        <v>0.52</v>
       </c>
       <c r="O78" t="n">
-        <v>7.619999999999999</v>
+        <v>0.7615</v>
       </c>
       <c r="P78" t="n">
         <v>1</v>
@@ -5788,19 +5788,19 @@
         </is>
       </c>
       <c r="K79" t="n">
-        <v>9.09</v>
+        <v>0.91</v>
       </c>
       <c r="L79" t="n">
-        <v>7.29</v>
+        <v>0.73</v>
       </c>
       <c r="M79" t="n">
-        <v>6.29</v>
+        <v>0.63</v>
       </c>
       <c r="N79" t="n">
-        <v>4.78</v>
+        <v>0.48</v>
       </c>
       <c r="O79" t="n">
-        <v>7.253499999999999</v>
+        <v>0.7264999999999999</v>
       </c>
       <c r="P79" t="n">
         <v>3</v>
@@ -5856,19 +5856,19 @@
         </is>
       </c>
       <c r="K80" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L80" t="n">
-        <v>9.869999999999999</v>
+        <v>0.99</v>
       </c>
       <c r="M80" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N80" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O80" t="n">
-        <v>9.954499999999999</v>
+        <v>0.9965000000000001</v>
       </c>
       <c r="P80" t="n">
         <v>1</v>
@@ -5924,19 +5924,19 @@
         </is>
       </c>
       <c r="K81" t="n">
-        <v>8.869999999999999</v>
+        <v>0.89</v>
       </c>
       <c r="L81" t="n">
-        <v>9.869999999999999</v>
+        <v>0.99</v>
       </c>
       <c r="M81" t="n">
-        <v>7.83</v>
+        <v>0.78</v>
       </c>
       <c r="N81" t="n">
-        <v>6.69</v>
+        <v>0.67</v>
       </c>
       <c r="O81" t="n">
-        <v>8.684999999999999</v>
+        <v>0.87</v>
       </c>
       <c r="P81" t="n">
         <v>2</v>
@@ -5992,19 +5992,19 @@
         </is>
       </c>
       <c r="K82" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L82" t="n">
-        <v>9.93</v>
+        <v>0.99</v>
       </c>
       <c r="M82" t="n">
-        <v>2.08</v>
+        <v>0.21</v>
       </c>
       <c r="N82" t="n">
-        <v>2.7</v>
+        <v>0.27</v>
       </c>
       <c r="O82" t="n">
-        <v>7.296500000000001</v>
+        <v>0.729</v>
       </c>
       <c r="P82" t="n">
         <v>3</v>
@@ -6060,19 +6060,19 @@
         </is>
       </c>
       <c r="K83" t="n">
-        <v>7.15</v>
+        <v>0.71</v>
       </c>
       <c r="L83" t="n">
-        <v>1.86</v>
+        <v>0.19</v>
       </c>
       <c r="M83" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N83" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O83" t="n">
-        <v>6.296</v>
+        <v>0.6294999999999999</v>
       </c>
       <c r="P83" t="n">
         <v>1</v>
@@ -6131,16 +6131,16 @@
         <v>0</v>
       </c>
       <c r="L84" t="n">
-        <v>1.86</v>
+        <v>0.19</v>
       </c>
       <c r="M84" t="n">
-        <v>7.29</v>
+        <v>0.73</v>
       </c>
       <c r="N84" t="n">
-        <v>6.04</v>
+        <v>0.6</v>
       </c>
       <c r="O84" t="n">
-        <v>3.015</v>
+        <v>0.3025</v>
       </c>
       <c r="P84" t="n">
         <v>3</v>
@@ -6196,19 +6196,19 @@
         </is>
       </c>
       <c r="K85" t="n">
-        <v>7.15</v>
+        <v>0.71</v>
       </c>
       <c r="L85" t="n">
-        <v>1.86</v>
+        <v>0.19</v>
       </c>
       <c r="M85" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.09</v>
       </c>
       <c r="N85" t="n">
-        <v>1.61</v>
+        <v>0.16</v>
       </c>
       <c r="O85" t="n">
-        <v>3.2255</v>
+        <v>0.3215</v>
       </c>
       <c r="P85" t="n">
         <v>2</v>
@@ -6264,19 +6264,19 @@
         </is>
       </c>
       <c r="K86" t="n">
-        <v>4.76</v>
+        <v>0.48</v>
       </c>
       <c r="L86" t="n">
-        <v>7.14</v>
+        <v>0.71</v>
       </c>
       <c r="M86" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N86" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O86" t="n">
-        <v>7.427</v>
+        <v>0.7425</v>
       </c>
       <c r="P86" t="n">
         <v>2</v>
@@ -6332,19 +6332,19 @@
         </is>
       </c>
       <c r="K87" t="n">
-        <v>9.029999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="L87" t="n">
-        <v>7.14</v>
+        <v>0.71</v>
       </c>
       <c r="M87" t="n">
-        <v>7.09</v>
+        <v>0.71</v>
       </c>
       <c r="N87" t="n">
-        <v>5.81</v>
+        <v>0.58</v>
       </c>
       <c r="O87" t="n">
-        <v>7.4975</v>
+        <v>0.7474999999999999</v>
       </c>
       <c r="P87" t="n">
         <v>1</v>
@@ -6400,19 +6400,19 @@
         </is>
       </c>
       <c r="K88" t="n">
-        <v>9.029999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="L88" t="n">
-        <v>7.37</v>
+        <v>0.74</v>
       </c>
       <c r="M88" t="n">
-        <v>4.28</v>
+        <v>0.43</v>
       </c>
       <c r="N88" t="n">
-        <v>1.51</v>
+        <v>0.15</v>
       </c>
       <c r="O88" t="n">
-        <v>6.370999999999999</v>
+        <v>0.6375</v>
       </c>
       <c r="P88" t="n">
         <v>3</v>
@@ -6468,19 +6468,19 @@
         </is>
       </c>
       <c r="K89" t="n">
-        <v>9.94</v>
+        <v>0.99</v>
       </c>
       <c r="L89" t="n">
-        <v>9.56</v>
+        <v>0.96</v>
       </c>
       <c r="M89" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N89" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O89" t="n">
-        <v>9.827999999999999</v>
+        <v>0.983</v>
       </c>
       <c r="P89" t="n">
         <v>1</v>
@@ -6536,19 +6536,19 @@
         </is>
       </c>
       <c r="K90" t="n">
-        <v>9.94</v>
+        <v>0.99</v>
       </c>
       <c r="L90" t="n">
-        <v>9.640000000000001</v>
+        <v>0.96</v>
       </c>
       <c r="M90" t="n">
-        <v>5.82</v>
+        <v>0.58</v>
       </c>
       <c r="N90" t="n">
-        <v>5.81</v>
+        <v>0.58</v>
       </c>
       <c r="O90" t="n">
-        <v>8.391499999999999</v>
+        <v>0.836</v>
       </c>
       <c r="P90" t="n">
         <v>2</v>
@@ -6604,19 +6604,19 @@
         </is>
       </c>
       <c r="K91" t="n">
-        <v>9.94</v>
+        <v>0.99</v>
       </c>
       <c r="L91" t="n">
-        <v>9.56</v>
+        <v>0.96</v>
       </c>
       <c r="M91" t="n">
-        <v>4.71</v>
+        <v>0.47</v>
       </c>
       <c r="N91" t="n">
-        <v>2.95</v>
+        <v>0.3</v>
       </c>
       <c r="O91" t="n">
-        <v>7.712499999999999</v>
+        <v>0.772</v>
       </c>
       <c r="P91" t="n">
         <v>3</v>
@@ -6672,19 +6672,19 @@
         </is>
       </c>
       <c r="K92" t="n">
-        <v>6.93</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L92" t="n">
-        <v>1.24</v>
+        <v>0.12</v>
       </c>
       <c r="M92" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N92" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O92" t="n">
-        <v>6.013</v>
+        <v>0.599</v>
       </c>
       <c r="P92" t="n">
         <v>1</v>
@@ -6743,16 +6743,16 @@
         <v>0</v>
       </c>
       <c r="L93" t="n">
-        <v>1.24</v>
+        <v>0.12</v>
       </c>
       <c r="M93" t="n">
-        <v>6.29</v>
+        <v>0.63</v>
       </c>
       <c r="N93" t="n">
-        <v>4.86</v>
+        <v>0.49</v>
       </c>
       <c r="O93" t="n">
-        <v>2.421</v>
+        <v>0.2415</v>
       </c>
       <c r="P93" t="n">
         <v>3</v>
@@ -6808,19 +6808,19 @@
         </is>
       </c>
       <c r="K94" t="n">
-        <v>6.93</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L94" t="n">
-        <v>1.84</v>
+        <v>0.18</v>
       </c>
       <c r="M94" t="n">
-        <v>2.86</v>
+        <v>0.29</v>
       </c>
       <c r="N94" t="n">
-        <v>2.63</v>
+        <v>0.26</v>
       </c>
       <c r="O94" t="n">
-        <v>3.6895</v>
+        <v>0.367</v>
       </c>
       <c r="P94" t="n">
         <v>2</v>
@@ -6876,19 +6876,19 @@
         </is>
       </c>
       <c r="K95" t="n">
-        <v>5.15</v>
+        <v>0.51</v>
       </c>
       <c r="L95" t="n">
-        <v>2.79</v>
+        <v>0.28</v>
       </c>
       <c r="M95" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N95" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O95" t="n">
-        <v>6.0215</v>
+        <v>0.601</v>
       </c>
       <c r="P95" t="n">
         <v>1</v>
@@ -6944,19 +6944,19 @@
         </is>
       </c>
       <c r="K96" t="n">
-        <v>5.15</v>
+        <v>0.51</v>
       </c>
       <c r="L96" t="n">
-        <v>2.79</v>
+        <v>0.28</v>
       </c>
       <c r="M96" t="n">
-        <v>7.29</v>
+        <v>0.73</v>
       </c>
       <c r="N96" t="n">
-        <v>6.04</v>
+        <v>0.6</v>
       </c>
       <c r="O96" t="n">
-        <v>4.8855</v>
+        <v>0.487</v>
       </c>
       <c r="P96" t="n">
         <v>2</v>
@@ -7012,19 +7012,19 @@
         </is>
       </c>
       <c r="K97" t="n">
-        <v>5.15</v>
+        <v>0.51</v>
       </c>
       <c r="L97" t="n">
-        <v>2.79</v>
+        <v>0.28</v>
       </c>
       <c r="M97" t="n">
-        <v>3.36</v>
+        <v>0.34</v>
       </c>
       <c r="N97" t="n">
-        <v>3.11</v>
+        <v>0.31</v>
       </c>
       <c r="O97" t="n">
-        <v>3.66</v>
+        <v>0.3655</v>
       </c>
       <c r="P97" t="n">
         <v>3</v>
@@ -7080,19 +7080,19 @@
         </is>
       </c>
       <c r="K98" t="n">
-        <v>8.630000000000001</v>
+        <v>0.86</v>
       </c>
       <c r="L98" t="n">
-        <v>5.58</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M98" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N98" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O98" t="n">
-        <v>8.042</v>
+        <v>0.804</v>
       </c>
       <c r="P98" t="n">
         <v>1</v>
@@ -7148,19 +7148,19 @@
         </is>
       </c>
       <c r="K99" t="n">
-        <v>8.630000000000001</v>
+        <v>0.86</v>
       </c>
       <c r="L99" t="n">
-        <v>5.58</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M99" t="n">
-        <v>5.21</v>
+        <v>0.52</v>
       </c>
       <c r="N99" t="n">
-        <v>4.64</v>
+        <v>0.35</v>
       </c>
       <c r="O99" t="n">
-        <v>6.279999999999999</v>
+        <v>0.6105</v>
       </c>
       <c r="P99" t="n">
         <v>3</v>
@@ -7216,19 +7216,19 @@
         </is>
       </c>
       <c r="K100" t="n">
-        <v>8.630000000000001</v>
+        <v>0.86</v>
       </c>
       <c r="L100" t="n">
-        <v>5.58</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="M100" t="n">
-        <v>7.83</v>
+        <v>0.78</v>
       </c>
       <c r="N100" t="n">
-        <v>5.71</v>
+        <v>0.57</v>
       </c>
       <c r="O100" t="n">
-        <v>6.964499999999999</v>
+        <v>0.6955000000000001</v>
       </c>
       <c r="P100" t="n">
         <v>2</v>
@@ -7284,19 +7284,19 @@
         </is>
       </c>
       <c r="K101" t="n">
-        <v>7.91</v>
+        <v>0.79</v>
       </c>
       <c r="L101" t="n">
-        <v>3.41</v>
+        <v>0.34</v>
       </c>
       <c r="M101" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N101" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O101" t="n">
-        <v>7.0665</v>
+        <v>0.7060000000000001</v>
       </c>
       <c r="P101" t="n">
         <v>1</v>
@@ -7352,19 +7352,19 @@
         </is>
       </c>
       <c r="K102" t="n">
-        <v>7.91</v>
+        <v>0.79</v>
       </c>
       <c r="L102" t="n">
-        <v>3.41</v>
+        <v>0.34</v>
       </c>
       <c r="M102" t="n">
-        <v>5.69</v>
+        <v>0.57</v>
       </c>
       <c r="N102" t="n">
-        <v>5.67</v>
+        <v>0.57</v>
       </c>
       <c r="O102" t="n">
-        <v>5.555</v>
+        <v>0.5555</v>
       </c>
       <c r="P102" t="n">
         <v>2</v>
@@ -7420,19 +7420,19 @@
         </is>
       </c>
       <c r="K103" t="n">
-        <v>7.91</v>
+        <v>0.79</v>
       </c>
       <c r="L103" t="n">
-        <v>3.88</v>
+        <v>0.39</v>
       </c>
       <c r="M103" t="n">
-        <v>1.24</v>
+        <v>0.12</v>
       </c>
       <c r="N103" t="n">
-        <v>2.47</v>
+        <v>0.25</v>
       </c>
       <c r="O103" t="n">
-        <v>4.3495</v>
+        <v>0.4349999999999999</v>
       </c>
       <c r="P103" t="n">
         <v>3</v>
@@ -7488,19 +7488,19 @@
         </is>
       </c>
       <c r="K104" t="n">
-        <v>9.199999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="L104" t="n">
-        <v>7.6</v>
+        <v>0.76</v>
       </c>
       <c r="M104" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N104" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O104" t="n">
-        <v>8.92</v>
+        <v>0.892</v>
       </c>
       <c r="P104" t="n">
         <v>1</v>
@@ -7556,19 +7556,19 @@
         </is>
       </c>
       <c r="K105" t="n">
-        <v>5.46</v>
+        <v>0.55</v>
       </c>
       <c r="L105" t="n">
-        <v>7.6</v>
+        <v>0.76</v>
       </c>
       <c r="M105" t="n">
-        <v>7.09</v>
+        <v>0.71</v>
       </c>
       <c r="N105" t="n">
-        <v>5.81</v>
+        <v>0.58</v>
       </c>
       <c r="O105" t="n">
-        <v>6.5875</v>
+        <v>0.6599999999999999</v>
       </c>
       <c r="P105" t="n">
         <v>3</v>
@@ -7624,19 +7624,19 @@
         </is>
       </c>
       <c r="K106" t="n">
-        <v>9.199999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="L106" t="n">
-        <v>7.8</v>
+        <v>0.78</v>
       </c>
       <c r="M106" t="n">
-        <v>5.73</v>
+        <v>0.57</v>
       </c>
       <c r="N106" t="n">
-        <v>2.89</v>
+        <v>0.29</v>
       </c>
       <c r="O106" t="n">
-        <v>7.0695</v>
+        <v>0.7064999999999999</v>
       </c>
       <c r="P106" t="n">
         <v>2</v>

</xml_diff>